<commit_message>
Save working project state from new_branch_07_05
</commit_message>
<xml_diff>
--- a/input/excel/T23_000000_t10Ved14.xlsx
+++ b/input/excel/T23_000000_t10Ved14.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="396" yWindow="36" windowWidth="8448" windowHeight="4872" tabRatio="359"/>
+    <workbookView xWindow="390" yWindow="30" windowWidth="8445" windowHeight="4875" tabRatio="359"/>
   </bookViews>
   <sheets>
     <sheet name="T10" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="139">
   <si>
     <t>тыс.руб.</t>
   </si>
@@ -95,15 +95,6 @@
     <t>денежные средства и денежные эквиваленты</t>
   </si>
   <si>
-    <t>Оборотные активы за 2023 год</t>
-  </si>
-  <si>
-    <t>Камчатский край</t>
-  </si>
-  <si>
-    <t>Организации без субъектов малого предпринимательства (1-этап)</t>
-  </si>
-  <si>
     <t>Всего по обследуемым видам экономической деятельности</t>
   </si>
   <si>
@@ -468,13 +459,16 @@
   </si>
   <si>
     <t>S</t>
+  </si>
+  <si>
+    <t>убрала название таблицы</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial Cyr"/>
@@ -537,6 +531,12 @@
       <b/>
       <sz val="10"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman CYR"/>
       <family val="1"/>
       <charset val="204"/>
     </font>
@@ -678,9 +678,6 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -689,9 +686,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -704,60 +698,6 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -783,6 +723,66 @@
     </xf>
     <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1090,91 +1090,81 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:R70"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="16" customWidth="1"/>
-    <col min="2" max="2" width="28.77734375" style="11" customWidth="1"/>
-    <col min="3" max="6" width="12.77734375" style="2" customWidth="1"/>
-    <col min="7" max="10" width="12.109375" style="2" customWidth="1"/>
-    <col min="11" max="16" width="12.88671875" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="10.7109375" style="14" customWidth="1"/>
+    <col min="2" max="2" width="28.7109375" style="10" customWidth="1"/>
+    <col min="3" max="6" width="12.7109375" style="2" customWidth="1"/>
+    <col min="7" max="10" width="12.140625" style="2" customWidth="1"/>
+    <col min="11" max="16" width="12.85546875" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="4" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15"/>
-      <c r="B1" s="11"/>
-      <c r="C1" s="27" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
+    <row r="1" spans="1:18" s="4" customFormat="1" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="13"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
-      <c r="K1" s="27" t="s">
-        <v>16</v>
-      </c>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="13"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="11"/>
       <c r="Q1" s="5"/>
       <c r="R1" s="5"/>
     </row>
-    <row r="2" spans="1:18" s="4" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
+    <row r="2" spans="1:18" s="4" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="13"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="D2" s="26"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
-      <c r="K2" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="14"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="12"/>
       <c r="Q2" s="5"/>
       <c r="R2" s="5"/>
     </row>
-    <row r="3" spans="1:18" s="4" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="18"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
+    <row r="3" spans="1:18" s="4" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="13"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
-      <c r="K3" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
-      <c r="O3" s="26"/>
-      <c r="P3" s="14"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="27"/>
+      <c r="M3" s="27"/>
+      <c r="N3" s="27"/>
+      <c r="O3" s="27"/>
+      <c r="P3" s="12"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
     </row>
-    <row r="4" spans="1:18" s="4" customFormat="1" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="11"/>
+    <row r="4" spans="1:18" s="4" customFormat="1" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="13"/>
+      <c r="B4" s="10"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -1189,92 +1179,92 @@
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
-      <c r="O4" s="25" t="s">
+      <c r="O4" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="P4" s="25"/>
+      <c r="P4" s="38"/>
       <c r="Q4" s="5"/>
       <c r="R4" s="5"/>
     </row>
-    <row r="5" spans="1:18" s="4" customFormat="1" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:18" s="4" customFormat="1" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="23" t="s">
+      <c r="D5" s="30"/>
+      <c r="E5" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="24"/>
-      <c r="J5" s="24"/>
-      <c r="K5" s="23" t="s">
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="L5" s="24"/>
-      <c r="M5" s="24"/>
-      <c r="N5" s="24"/>
-      <c r="O5" s="24"/>
-      <c r="P5" s="24"/>
-    </row>
-    <row r="6" spans="1:18" s="4" customFormat="1" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="23" t="s">
+      <c r="L5" s="30"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="30"/>
+      <c r="O5" s="30"/>
+      <c r="P5" s="30"/>
+    </row>
+    <row r="6" spans="1:18" s="4" customFormat="1" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="39"/>
+      <c r="B6" s="42"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="24"/>
-      <c r="G6" s="28" t="s">
+      <c r="F6" s="30"/>
+      <c r="G6" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="29"/>
-      <c r="I6" s="28" t="s">
+      <c r="H6" s="32"/>
+      <c r="I6" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="32"/>
-      <c r="K6" s="23" t="s">
+      <c r="J6" s="35"/>
+      <c r="K6" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="L6" s="24"/>
-      <c r="M6" s="23" t="s">
+      <c r="L6" s="30"/>
+      <c r="M6" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="N6" s="24"/>
-      <c r="O6" s="23" t="s">
+      <c r="N6" s="30"/>
+      <c r="O6" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="P6" s="24"/>
-    </row>
-    <row r="7" spans="1:18" s="4" customFormat="1" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="17"/>
-      <c r="B7" s="21"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="30"/>
-      <c r="H7" s="31"/>
-      <c r="I7" s="33"/>
-      <c r="J7" s="34"/>
-      <c r="K7" s="24"/>
-      <c r="L7" s="24"/>
-      <c r="M7" s="24"/>
-      <c r="N7" s="24"/>
-      <c r="O7" s="24"/>
-      <c r="P7" s="24"/>
-    </row>
-    <row r="8" spans="1:18" s="4" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17"/>
-      <c r="B8" s="22"/>
+      <c r="P6" s="30"/>
+    </row>
+    <row r="7" spans="1:18" s="4" customFormat="1" ht="28.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="39"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="37"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="30"/>
+      <c r="M7" s="30"/>
+      <c r="N7" s="30"/>
+      <c r="O7" s="30"/>
+      <c r="P7" s="30"/>
+    </row>
+    <row r="8" spans="1:18" s="4" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="39"/>
+      <c r="B8" s="43"/>
       <c r="C8" s="6" t="s">
         <v>12</v>
       </c>
@@ -1318,132 +1308,132 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:18" s="10" customFormat="1" ht="10.199999999999999" x14ac:dyDescent="0.2">
-      <c r="A9" s="8" t="s">
+    <row r="9" spans="1:18" s="9" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A9" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="8">
         <v>1</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="8">
         <v>2</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="8">
         <v>3</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="8">
         <v>4</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="8">
         <v>5</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="8">
         <v>6</v>
       </c>
-      <c r="I9" s="9">
+      <c r="I9" s="8">
         <v>7</v>
       </c>
-      <c r="J9" s="9">
+      <c r="J9" s="8">
         <v>8</v>
       </c>
-      <c r="K9" s="9">
+      <c r="K9" s="8">
         <v>9</v>
       </c>
-      <c r="L9" s="9">
+      <c r="L9" s="8">
         <v>10</v>
       </c>
-      <c r="M9" s="9">
+      <c r="M9" s="8">
         <v>11</v>
       </c>
-      <c r="N9" s="9">
+      <c r="N9" s="8">
         <v>12</v>
       </c>
-      <c r="O9" s="9">
+      <c r="O9" s="8">
         <v>13</v>
       </c>
-      <c r="P9" s="9">
+      <c r="P9" s="8">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:18" s="39" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="36" t="s">
-        <v>120</v>
-      </c>
-      <c r="B10" s="37"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="38"/>
-      <c r="G10" s="38"/>
-      <c r="H10" s="38"/>
-      <c r="I10" s="38"/>
-      <c r="J10" s="38"/>
-      <c r="K10" s="38"/>
-      <c r="L10" s="38"/>
-      <c r="M10" s="38"/>
-      <c r="N10" s="38"/>
-      <c r="O10" s="38"/>
-      <c r="P10" s="38"/>
-    </row>
-    <row r="11" spans="1:18" s="39" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A11" s="36" t="s">
-        <v>121</v>
-      </c>
-      <c r="B11" s="40" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="38">
+    <row r="10" spans="1:18" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="B10" s="17"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="18"/>
+      <c r="N10" s="18"/>
+      <c r="O10" s="18"/>
+      <c r="P10" s="18"/>
+    </row>
+    <row r="11" spans="1:18" s="19" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A11" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="18">
         <v>250446609</v>
       </c>
-      <c r="D11" s="38">
+      <c r="D11" s="18">
         <v>318620610</v>
       </c>
-      <c r="E11" s="38">
+      <c r="E11" s="18">
         <v>66760265</v>
       </c>
-      <c r="F11" s="38">
+      <c r="F11" s="18">
         <v>77715920</v>
       </c>
-      <c r="G11" s="38">
+      <c r="G11" s="18">
         <v>879305</v>
       </c>
-      <c r="H11" s="38">
+      <c r="H11" s="18">
         <v>1623558</v>
       </c>
-      <c r="I11" s="38">
+      <c r="I11" s="18">
         <v>107038823</v>
       </c>
-      <c r="J11" s="38">
+      <c r="J11" s="18">
         <v>115644676</v>
       </c>
-      <c r="K11" s="38">
+      <c r="K11" s="18">
         <v>16020827</v>
       </c>
-      <c r="L11" s="38">
+      <c r="L11" s="18">
         <v>18562758</v>
       </c>
-      <c r="M11" s="38">
+      <c r="M11" s="18">
         <v>51711258</v>
       </c>
-      <c r="N11" s="38">
+      <c r="N11" s="18">
         <v>79714976</v>
       </c>
-      <c r="O11" s="38">
+      <c r="O11" s="18">
         <v>8036131</v>
       </c>
-      <c r="P11" s="38">
+      <c r="P11" s="18">
         <v>25358722</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="35" t="s">
-        <v>21</v>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A12" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>18</v>
       </c>
       <c r="C12" s="2">
         <v>83430857</v>
@@ -1488,62 +1478,62 @@
         <v>6528516</v>
       </c>
     </row>
-    <row r="13" spans="1:18" s="39" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
-      <c r="A13" s="36" t="s">
-        <v>122</v>
-      </c>
-      <c r="B13" s="40" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" s="38">
+    <row r="13" spans="1:18" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A13" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="18">
         <v>105936412</v>
       </c>
-      <c r="D13" s="38">
+      <c r="D13" s="18">
         <v>164347190</v>
       </c>
-      <c r="E13" s="38">
+      <c r="E13" s="18">
         <v>27102831</v>
       </c>
-      <c r="F13" s="38">
+      <c r="F13" s="18">
         <v>29271082</v>
       </c>
-      <c r="G13" s="38">
+      <c r="G13" s="18">
         <v>80687</v>
       </c>
-      <c r="H13" s="38">
+      <c r="H13" s="18">
         <v>145586</v>
       </c>
-      <c r="I13" s="38">
+      <c r="I13" s="18">
         <v>36909780</v>
       </c>
-      <c r="J13" s="38">
+      <c r="J13" s="18">
         <v>52628064</v>
       </c>
-      <c r="K13" s="38">
+      <c r="K13" s="18">
         <v>10905203</v>
       </c>
-      <c r="L13" s="38">
+      <c r="L13" s="18">
         <v>10681119</v>
       </c>
-      <c r="M13" s="38">
+      <c r="M13" s="18">
         <v>30127456</v>
       </c>
-      <c r="N13" s="38">
+      <c r="N13" s="18">
         <v>54097850</v>
       </c>
-      <c r="O13" s="38">
+      <c r="O13" s="18">
         <v>810455</v>
       </c>
-      <c r="P13" s="38">
+      <c r="P13" s="18">
         <v>17523489</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="52.8" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="35" t="s">
-        <v>24</v>
+    <row r="14" spans="1:18" ht="51" x14ac:dyDescent="0.2">
+      <c r="A14" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>21</v>
       </c>
       <c r="C14" s="2">
         <v>1955545</v>
@@ -1588,12 +1578,12 @@
         <v>32735</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="35" t="s">
-        <v>26</v>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A15" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>23</v>
       </c>
       <c r="C15" s="2">
         <v>103980867</v>
@@ -1638,62 +1628,62 @@
         <v>17490754</v>
       </c>
     </row>
-    <row r="16" spans="1:18" s="39" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A16" s="36" t="s">
-        <v>123</v>
-      </c>
-      <c r="B16" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="38">
+    <row r="16" spans="1:18" s="19" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A16" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="18">
         <v>33466860</v>
       </c>
-      <c r="D16" s="38">
+      <c r="D16" s="18">
         <v>27491671</v>
       </c>
-      <c r="E16" s="38">
+      <c r="E16" s="18">
         <v>12944689</v>
       </c>
-      <c r="F16" s="38">
+      <c r="F16" s="18">
         <v>15607540</v>
       </c>
-      <c r="G16" s="38">
+      <c r="G16" s="18">
         <v>99828</v>
       </c>
-      <c r="H16" s="38">
+      <c r="H16" s="18">
         <v>10650</v>
       </c>
-      <c r="I16" s="38">
+      <c r="I16" s="18">
         <v>16054072</v>
       </c>
-      <c r="J16" s="38">
+      <c r="J16" s="18">
         <v>8650720</v>
       </c>
-      <c r="K16" s="38">
+      <c r="K16" s="18">
         <v>62000</v>
       </c>
-      <c r="L16" s="38">
+      <c r="L16" s="18">
         <v>677383</v>
       </c>
-      <c r="M16" s="38">
+      <c r="M16" s="18">
         <v>2391347</v>
       </c>
-      <c r="N16" s="38">
+      <c r="N16" s="18">
         <v>139261</v>
       </c>
-      <c r="O16" s="38">
+      <c r="O16" s="18">
         <v>1914924</v>
       </c>
-      <c r="P16" s="38">
+      <c r="P16" s="18">
         <v>2406117</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="35" t="s">
-        <v>29</v>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A17" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>26</v>
       </c>
       <c r="C17" s="2">
         <v>33466860</v>
@@ -1738,62 +1728,62 @@
         <v>2406117</v>
       </c>
     </row>
-    <row r="18" spans="1:16" s="39" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A18" s="36" t="s">
-        <v>124</v>
-      </c>
-      <c r="B18" s="40" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="38">
+    <row r="18" spans="1:16" s="19" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A18" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="B18" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="18">
         <v>21052953</v>
       </c>
-      <c r="D18" s="38">
+      <c r="D18" s="18">
         <v>22948469</v>
       </c>
-      <c r="E18" s="38">
+      <c r="E18" s="18">
         <v>4590465</v>
       </c>
-      <c r="F18" s="38">
+      <c r="F18" s="18">
         <v>5695784</v>
       </c>
-      <c r="G18" s="38">
+      <c r="G18" s="18">
         <v>18370</v>
       </c>
-      <c r="H18" s="38">
+      <c r="H18" s="18">
         <v>152761</v>
       </c>
-      <c r="I18" s="38">
+      <c r="I18" s="18">
         <v>6918321</v>
       </c>
-      <c r="J18" s="38">
+      <c r="J18" s="18">
         <v>8239073</v>
       </c>
-      <c r="K18" s="38">
+      <c r="K18" s="18">
         <v>2363761</v>
       </c>
-      <c r="L18" s="38">
+      <c r="L18" s="18">
         <v>2044762</v>
       </c>
-      <c r="M18" s="38">
+      <c r="M18" s="18">
         <v>3781149</v>
       </c>
-      <c r="N18" s="38">
+      <c r="N18" s="18">
         <v>3680196</v>
       </c>
-      <c r="O18" s="38">
+      <c r="O18" s="18">
         <v>3380887</v>
       </c>
-      <c r="P18" s="38">
+      <c r="P18" s="18">
         <v>3135893</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A19" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="35" t="s">
-        <v>32</v>
+    <row r="19" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A19" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="C19" s="2">
         <v>15245469</v>
@@ -1838,12 +1828,12 @@
         <v>152552</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20" s="35" t="s">
-        <v>34</v>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A20" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>31</v>
       </c>
       <c r="C20" s="2">
         <v>422422</v>
@@ -1858,10 +1848,10 @@
         <v>135323</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I20" s="2">
         <v>146122</v>
@@ -1870,7 +1860,7 @@
         <v>126855</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L20" s="2">
         <v>51196</v>
@@ -1882,18 +1872,18 @@
         <v>197543</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P20" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" ht="66" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="B21" s="35" t="s">
-        <v>37</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>34</v>
       </c>
       <c r="C21" s="2">
         <v>47</v>
@@ -1902,34 +1892,34 @@
         <v>47</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="O21" s="2">
         <v>47</v>
@@ -1938,12 +1928,12 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="B22" s="35" t="s">
-        <v>39</v>
+    <row r="22" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A22" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>36</v>
       </c>
       <c r="C22" s="2">
         <v>24489</v>
@@ -1958,10 +1948,10 @@
         <v>20296</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I22" s="2">
         <v>3183</v>
@@ -1970,10 +1960,10 @@
         <v>2229</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M22" s="2">
         <v>2299</v>
@@ -1988,12 +1978,12 @@
         <v>144</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A23" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="35" t="s">
-        <v>41</v>
+    <row r="23" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A23" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>38</v>
       </c>
       <c r="C23" s="2">
         <v>5360526</v>
@@ -2020,7 +2010,7 @@
         <v>690478</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L23" s="2">
         <v>19650</v>
@@ -2038,62 +2028,62 @@
         <v>2983150</v>
       </c>
     </row>
-    <row r="24" spans="1:16" s="39" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
-      <c r="A24" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="B24" s="40" t="s">
-        <v>42</v>
-      </c>
-      <c r="C24" s="38">
+    <row r="24" spans="1:16" s="19" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A24" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="B24" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" s="18">
         <v>26961006</v>
       </c>
-      <c r="D24" s="38">
+      <c r="D24" s="18">
         <v>29542714</v>
       </c>
-      <c r="E24" s="38">
+      <c r="E24" s="18">
         <v>7659260</v>
       </c>
-      <c r="F24" s="38">
+      <c r="F24" s="18">
         <v>8078103</v>
       </c>
-      <c r="G24" s="38">
+      <c r="G24" s="18">
         <v>20277</v>
       </c>
-      <c r="H24" s="38">
+      <c r="H24" s="18">
         <v>19447</v>
       </c>
-      <c r="I24" s="38">
+      <c r="I24" s="18">
         <v>11727886</v>
       </c>
-      <c r="J24" s="38">
+      <c r="J24" s="18">
         <v>14374616</v>
       </c>
-      <c r="K24" s="38">
+      <c r="K24" s="18">
         <v>867379</v>
       </c>
-      <c r="L24" s="38">
+      <c r="L24" s="18">
         <v>835900</v>
       </c>
-      <c r="M24" s="38">
+      <c r="M24" s="18">
         <v>5658447</v>
       </c>
-      <c r="N24" s="38">
+      <c r="N24" s="18">
         <v>5255744</v>
       </c>
-      <c r="O24" s="38">
+      <c r="O24" s="18">
         <v>1027757</v>
       </c>
-      <c r="P24" s="38">
+      <c r="P24" s="18">
         <v>978904</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A25" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="B25" s="35" t="s">
-        <v>44</v>
+    <row r="25" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A25" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>41</v>
       </c>
       <c r="C25" s="2">
         <v>26961006</v>
@@ -2138,62 +2128,62 @@
         <v>978904</v>
       </c>
     </row>
-    <row r="26" spans="1:16" s="39" customFormat="1" ht="92.4" x14ac:dyDescent="0.25">
-      <c r="A26" s="36" t="s">
-        <v>126</v>
-      </c>
-      <c r="B26" s="40" t="s">
-        <v>45</v>
-      </c>
-      <c r="C26" s="38">
+    <row r="26" spans="1:16" s="19" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A26" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="18">
         <v>1950038</v>
       </c>
-      <c r="D26" s="38">
+      <c r="D26" s="18">
         <v>2340572</v>
       </c>
-      <c r="E26" s="38">
+      <c r="E26" s="18">
         <v>572496</v>
       </c>
-      <c r="F26" s="38">
+      <c r="F26" s="18">
         <v>655483</v>
       </c>
-      <c r="G26" s="38">
+      <c r="G26" s="18">
         <v>7865</v>
       </c>
-      <c r="H26" s="38">
+      <c r="H26" s="18">
         <v>3583</v>
       </c>
-      <c r="I26" s="38">
+      <c r="I26" s="18">
         <v>1147141</v>
       </c>
-      <c r="J26" s="38">
+      <c r="J26" s="18">
         <v>1415534</v>
       </c>
-      <c r="K26" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="L26" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M26" s="38">
+      <c r="K26" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="L26" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="M26" s="18">
         <v>167946</v>
       </c>
-      <c r="N26" s="38">
+      <c r="N26" s="18">
         <v>258370</v>
       </c>
-      <c r="O26" s="38">
+      <c r="O26" s="18">
         <v>54590</v>
       </c>
-      <c r="P26" s="38">
+      <c r="P26" s="18">
         <v>7602</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A27" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B27" s="35" t="s">
-        <v>47</v>
+    <row r="27" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A27" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>44</v>
       </c>
       <c r="C27" s="2">
         <v>1656817</v>
@@ -2220,10 +2210,10 @@
         <v>1158090</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M27" s="2">
         <v>164317</v>
@@ -2238,12 +2228,12 @@
         <v>2380</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="B28" s="35" t="s">
-        <v>49</v>
+    <row r="28" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A28" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>46</v>
       </c>
       <c r="C28" s="2">
         <v>293221</v>
@@ -2258,10 +2248,10 @@
         <v>35017</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I28" s="2">
         <v>263318</v>
@@ -2270,10 +2260,10 @@
         <v>257444</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M28" s="2">
         <v>3629</v>
@@ -2288,62 +2278,62 @@
         <v>5222</v>
       </c>
     </row>
-    <row r="29" spans="1:16" s="39" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="36" t="s">
-        <v>127</v>
-      </c>
-      <c r="B29" s="40" t="s">
-        <v>50</v>
-      </c>
-      <c r="C29" s="38">
+    <row r="29" spans="1:16" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="C29" s="18">
         <v>16433156</v>
       </c>
-      <c r="D29" s="38">
+      <c r="D29" s="18">
         <v>21998473</v>
       </c>
-      <c r="E29" s="38">
+      <c r="E29" s="18">
         <v>7224119</v>
       </c>
-      <c r="F29" s="38">
+      <c r="F29" s="18">
         <v>10483856</v>
       </c>
-      <c r="G29" s="38">
+      <c r="G29" s="18">
         <v>176934</v>
       </c>
-      <c r="H29" s="38">
+      <c r="H29" s="18">
         <v>598511</v>
       </c>
-      <c r="I29" s="38">
+      <c r="I29" s="18">
         <v>5948981</v>
       </c>
-      <c r="J29" s="38">
+      <c r="J29" s="18">
         <v>5136040</v>
       </c>
-      <c r="K29" s="38">
+      <c r="K29" s="18">
         <v>346289</v>
       </c>
-      <c r="L29" s="38">
+      <c r="L29" s="18">
         <v>818732</v>
       </c>
-      <c r="M29" s="38">
+      <c r="M29" s="18">
         <v>2625684</v>
       </c>
-      <c r="N29" s="38">
+      <c r="N29" s="18">
         <v>4851304</v>
       </c>
-      <c r="O29" s="38">
+      <c r="O29" s="18">
         <v>111149</v>
       </c>
-      <c r="P29" s="38">
+      <c r="P29" s="18">
         <v>110030</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A30" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="B30" s="35" t="s">
-        <v>52</v>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A30" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>49</v>
       </c>
       <c r="C30" s="2">
         <v>12127276</v>
@@ -2388,12 +2378,12 @@
         <v>87255</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="B31" s="35" t="s">
-        <v>54</v>
+    <row r="31" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A31" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>51</v>
       </c>
       <c r="C31" s="2">
         <v>4250141</v>
@@ -2408,10 +2398,10 @@
         <v>1693287</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I31" s="2">
         <v>1254608</v>
@@ -2438,12 +2428,12 @@
         <v>16804</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A32" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B32" s="35" t="s">
-        <v>56</v>
+    <row r="32" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A32" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>53</v>
       </c>
       <c r="C32" s="2">
         <v>55739</v>
@@ -2458,10 +2448,10 @@
         <v>38896</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I32" s="2">
         <v>7504</v>
@@ -2470,10 +2460,10 @@
         <v>1164</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M32" s="2">
         <v>4</v>
@@ -2488,62 +2478,62 @@
         <v>5971</v>
       </c>
     </row>
-    <row r="33" spans="1:16" s="39" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
-      <c r="A33" s="36" t="s">
-        <v>128</v>
-      </c>
-      <c r="B33" s="40" t="s">
-        <v>57</v>
-      </c>
-      <c r="C33" s="38">
+    <row r="33" spans="1:16" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A33" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="B33" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C33" s="18">
         <v>25181421</v>
       </c>
-      <c r="D33" s="38">
+      <c r="D33" s="18">
         <v>27074181</v>
       </c>
-      <c r="E33" s="38">
+      <c r="E33" s="18">
         <v>5119856</v>
       </c>
-      <c r="F33" s="38">
+      <c r="F33" s="18">
         <v>5668838</v>
       </c>
-      <c r="G33" s="38">
+      <c r="G33" s="18">
         <v>321624</v>
       </c>
-      <c r="H33" s="38">
+      <c r="H33" s="18">
         <v>527147</v>
       </c>
-      <c r="I33" s="38">
+      <c r="I33" s="18">
         <v>18206518</v>
       </c>
-      <c r="J33" s="38">
+      <c r="J33" s="18">
         <v>17331381</v>
       </c>
-      <c r="K33" s="38">
+      <c r="K33" s="18">
         <v>283008</v>
       </c>
-      <c r="L33" s="38">
+      <c r="L33" s="18">
         <v>1945653</v>
       </c>
-      <c r="M33" s="38">
+      <c r="M33" s="18">
         <v>713529</v>
       </c>
-      <c r="N33" s="38">
+      <c r="N33" s="18">
         <v>705275</v>
       </c>
-      <c r="O33" s="38">
+      <c r="O33" s="18">
         <v>536886</v>
       </c>
-      <c r="P33" s="38">
+      <c r="P33" s="18">
         <v>895887</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="B34" s="35" t="s">
-        <v>59</v>
+    <row r="34" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A34" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>56</v>
       </c>
       <c r="C34" s="2">
         <v>23187290</v>
@@ -2588,12 +2578,12 @@
         <v>891017</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B35" s="35" t="s">
-        <v>61</v>
+    <row r="35" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A35" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>58</v>
       </c>
       <c r="C35" s="2">
         <v>1994131</v>
@@ -2638,62 +2628,62 @@
         <v>4870</v>
       </c>
     </row>
-    <row r="36" spans="1:16" s="39" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A36" s="36" t="s">
-        <v>129</v>
-      </c>
-      <c r="B36" s="40" t="s">
-        <v>62</v>
-      </c>
-      <c r="C36" s="38">
+    <row r="36" spans="1:16" s="19" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A36" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="B36" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="18">
         <v>7718983</v>
       </c>
-      <c r="D36" s="38">
+      <c r="D36" s="18">
         <v>9648367</v>
       </c>
-      <c r="E36" s="38">
+      <c r="E36" s="18">
         <v>1107840</v>
       </c>
-      <c r="F36" s="38">
+      <c r="F36" s="18">
         <v>1600527</v>
       </c>
-      <c r="G36" s="38">
+      <c r="G36" s="18">
         <v>101235</v>
       </c>
-      <c r="H36" s="38">
+      <c r="H36" s="18">
         <v>97486</v>
       </c>
-      <c r="I36" s="38">
+      <c r="I36" s="18">
         <v>4927180</v>
       </c>
-      <c r="J36" s="38">
+      <c r="J36" s="18">
         <v>2997002</v>
       </c>
-      <c r="K36" s="38">
+      <c r="K36" s="18">
         <v>23203</v>
       </c>
-      <c r="L36" s="38">
+      <c r="L36" s="18">
         <v>3</v>
       </c>
-      <c r="M36" s="38">
+      <c r="M36" s="18">
         <v>1502251</v>
       </c>
-      <c r="N36" s="38">
+      <c r="N36" s="18">
         <v>4897150</v>
       </c>
-      <c r="O36" s="38">
+      <c r="O36" s="18">
         <v>57274</v>
       </c>
-      <c r="P36" s="38">
+      <c r="P36" s="18">
         <v>56199</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B37" s="35" t="s">
-        <v>64</v>
+    <row r="37" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A37" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>61</v>
       </c>
       <c r="C37" s="2">
         <v>54256</v>
@@ -2738,12 +2728,12 @@
         <v>453</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A38" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="B38" s="35" t="s">
-        <v>66</v>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A38" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>63</v>
       </c>
       <c r="C38" s="2">
         <v>997493</v>
@@ -2773,7 +2763,7 @@
         <v>23200</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M38" s="2">
         <v>2080</v>
@@ -2788,12 +2778,12 @@
         <v>1660</v>
       </c>
     </row>
-    <row r="39" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A39" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="B39" s="35" t="s">
-        <v>68</v>
+    <row r="39" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A39" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>65</v>
       </c>
       <c r="C39" s="2">
         <v>1227508</v>
@@ -2820,10 +2810,10 @@
         <v>544799</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M39" s="2">
         <v>244091</v>
@@ -2838,12 +2828,12 @@
         <v>975</v>
       </c>
     </row>
-    <row r="40" spans="1:16" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A40" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="B40" s="35" t="s">
-        <v>70</v>
+    <row r="40" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A40" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>67</v>
       </c>
       <c r="C40" s="2">
         <v>5439726</v>
@@ -2870,10 +2860,10 @@
         <v>1964249</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M40" s="2">
         <v>1254902</v>
@@ -2888,62 +2878,62 @@
         <v>53111</v>
       </c>
     </row>
-    <row r="41" spans="1:16" s="39" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
-      <c r="A41" s="36" t="s">
-        <v>130</v>
-      </c>
-      <c r="B41" s="40" t="s">
-        <v>71</v>
-      </c>
-      <c r="C41" s="38">
+    <row r="41" spans="1:16" s="19" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A41" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="B41" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="C41" s="18">
         <v>1605924</v>
       </c>
-      <c r="D41" s="38">
+      <c r="D41" s="18">
         <v>1613296</v>
       </c>
-      <c r="E41" s="38">
+      <c r="E41" s="18">
         <v>165460</v>
       </c>
-      <c r="F41" s="38">
+      <c r="F41" s="18">
         <v>197743</v>
       </c>
-      <c r="G41" s="38">
+      <c r="G41" s="18">
         <v>49075</v>
       </c>
-      <c r="H41" s="38">
+      <c r="H41" s="18">
         <v>64769</v>
       </c>
-      <c r="I41" s="38">
+      <c r="I41" s="18">
         <v>646127</v>
       </c>
-      <c r="J41" s="38">
+      <c r="J41" s="18">
         <v>554507</v>
       </c>
-      <c r="K41" s="38">
+      <c r="K41" s="18">
         <v>83075</v>
       </c>
-      <c r="L41" s="38">
+      <c r="L41" s="18">
         <v>217622</v>
       </c>
-      <c r="M41" s="38">
+      <c r="M41" s="18">
         <v>577560</v>
       </c>
-      <c r="N41" s="38">
+      <c r="N41" s="18">
         <v>421184</v>
       </c>
-      <c r="O41" s="38">
+      <c r="O41" s="18">
         <v>84627</v>
       </c>
-      <c r="P41" s="38">
+      <c r="P41" s="18">
         <v>157471</v>
       </c>
     </row>
-    <row r="42" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A42" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="B42" s="35" t="s">
-        <v>73</v>
+    <row r="42" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A42" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>70</v>
       </c>
       <c r="C42" s="2">
         <v>1605924</v>
@@ -2988,62 +2978,62 @@
         <v>157471</v>
       </c>
     </row>
-    <row r="43" spans="1:16" s="39" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A43" s="36" t="s">
-        <v>131</v>
-      </c>
-      <c r="B43" s="40" t="s">
-        <v>74</v>
-      </c>
-      <c r="C43" s="38">
+    <row r="43" spans="1:16" s="19" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A43" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="B43" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="C43" s="18">
         <v>3526</v>
       </c>
-      <c r="D43" s="38">
+      <c r="D43" s="18">
         <v>781</v>
       </c>
-      <c r="E43" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="F43" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="G43" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="H43" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="I43" s="38">
+      <c r="E43" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="F43" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="G43" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="H43" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="I43" s="18">
         <v>1367</v>
       </c>
-      <c r="J43" s="38">
+      <c r="J43" s="18">
         <v>764</v>
       </c>
-      <c r="K43" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="L43" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M43" s="38">
+      <c r="K43" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="L43" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="M43" s="18">
         <v>2159</v>
       </c>
-      <c r="N43" s="38">
+      <c r="N43" s="18">
         <v>17</v>
       </c>
-      <c r="O43" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="P43" s="38" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A44" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="B44" s="35" t="s">
-        <v>76</v>
+      <c r="O43" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="P43" s="18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A44" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C44" s="2">
         <v>3526</v>
@@ -3052,16 +3042,16 @@
         <v>781</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I44" s="2">
         <v>1367</v>
@@ -3070,10 +3060,10 @@
         <v>764</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M44" s="2">
         <v>2159</v>
@@ -3082,68 +3072,68 @@
         <v>17</v>
       </c>
       <c r="O44" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P44" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" s="39" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A45" s="36" t="s">
-        <v>132</v>
-      </c>
-      <c r="B45" s="40" t="s">
-        <v>77</v>
-      </c>
-      <c r="C45" s="38">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" s="19" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A45" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="B45" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="C45" s="18">
         <v>4366514</v>
       </c>
-      <c r="D45" s="38">
+      <c r="D45" s="18">
         <v>3948315</v>
       </c>
-      <c r="E45" s="38">
+      <c r="E45" s="18">
         <v>244</v>
       </c>
-      <c r="F45" s="38">
+      <c r="F45" s="18">
         <v>6780</v>
       </c>
-      <c r="G45" s="38">
+      <c r="G45" s="18">
         <v>73</v>
       </c>
-      <c r="H45" s="38">
+      <c r="H45" s="18">
         <v>76</v>
       </c>
-      <c r="I45" s="38">
+      <c r="I45" s="18">
         <v>1698664</v>
       </c>
-      <c r="J45" s="38">
+      <c r="J45" s="18">
         <v>449918</v>
       </c>
-      <c r="K45" s="38">
+      <c r="K45" s="18">
         <v>671532</v>
       </c>
-      <c r="L45" s="38">
+      <c r="L45" s="18">
         <v>728514</v>
       </c>
-      <c r="M45" s="38">
+      <c r="M45" s="18">
         <v>1976456</v>
       </c>
-      <c r="N45" s="38">
+      <c r="N45" s="18">
         <v>2744655</v>
       </c>
-      <c r="O45" s="38">
+      <c r="O45" s="18">
         <v>19545</v>
       </c>
-      <c r="P45" s="38">
+      <c r="P45" s="18">
         <v>18372</v>
       </c>
     </row>
-    <row r="46" spans="1:16" ht="52.8" x14ac:dyDescent="0.25">
-      <c r="A46" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="B46" s="35" t="s">
-        <v>79</v>
+    <row r="46" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+      <c r="A46" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="C46" s="2">
         <v>4366514</v>
@@ -3188,62 +3178,62 @@
         <v>18372</v>
       </c>
     </row>
-    <row r="47" spans="1:16" s="39" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
-      <c r="A47" s="36" t="s">
-        <v>133</v>
-      </c>
-      <c r="B47" s="40" t="s">
-        <v>80</v>
-      </c>
-      <c r="C47" s="38">
+    <row r="47" spans="1:16" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A47" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="B47" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="C47" s="18">
         <v>969471</v>
       </c>
-      <c r="D47" s="38">
+      <c r="D47" s="18">
         <v>1176865</v>
       </c>
-      <c r="E47" s="38">
+      <c r="E47" s="18">
         <v>30067</v>
       </c>
-      <c r="F47" s="38">
+      <c r="F47" s="18">
         <v>31194</v>
       </c>
-      <c r="G47" s="38">
+      <c r="G47" s="18">
         <v>1746</v>
       </c>
-      <c r="H47" s="38">
+      <c r="H47" s="18">
         <v>994</v>
       </c>
-      <c r="I47" s="38">
+      <c r="I47" s="18">
         <v>510140</v>
       </c>
-      <c r="J47" s="38">
+      <c r="J47" s="18">
         <v>542953</v>
       </c>
-      <c r="K47" s="38">
+      <c r="K47" s="18">
         <v>143639</v>
       </c>
-      <c r="L47" s="38">
+      <c r="L47" s="18">
         <v>323332</v>
       </c>
-      <c r="M47" s="38">
+      <c r="M47" s="18">
         <v>254618</v>
       </c>
-      <c r="N47" s="38">
+      <c r="N47" s="18">
         <v>248274</v>
       </c>
-      <c r="O47" s="38">
+      <c r="O47" s="18">
         <v>29261</v>
       </c>
-      <c r="P47" s="38">
+      <c r="P47" s="18">
         <v>30118</v>
       </c>
     </row>
-    <row r="48" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A48" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="B48" s="35" t="s">
-        <v>82</v>
+    <row r="48" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A48" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B48" s="15" t="s">
+        <v>79</v>
       </c>
       <c r="C48" s="2">
         <v>969471</v>
@@ -3288,62 +3278,62 @@
         <v>30118</v>
       </c>
     </row>
-    <row r="49" spans="1:16" s="39" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A49" s="36" t="s">
-        <v>134</v>
-      </c>
-      <c r="B49" s="40" t="s">
-        <v>83</v>
-      </c>
-      <c r="C49" s="38">
+    <row r="49" spans="1:16" s="19" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A49" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="B49" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="C49" s="18">
         <v>3965481</v>
       </c>
-      <c r="D49" s="38">
+      <c r="D49" s="18">
         <v>5536767</v>
       </c>
-      <c r="E49" s="38">
+      <c r="E49" s="18">
         <v>156739</v>
       </c>
-      <c r="F49" s="38">
+      <c r="F49" s="18">
         <v>270756</v>
       </c>
-      <c r="G49" s="38">
+      <c r="G49" s="18">
         <v>1490</v>
       </c>
-      <c r="H49" s="38">
+      <c r="H49" s="18">
         <v>2469</v>
       </c>
-      <c r="I49" s="38">
+      <c r="I49" s="18">
         <v>2223161</v>
       </c>
-      <c r="J49" s="38">
+      <c r="J49" s="18">
         <v>3141624</v>
       </c>
-      <c r="K49" s="38">
+      <c r="K49" s="18">
         <v>172138</v>
       </c>
-      <c r="L49" s="38">
+      <c r="L49" s="18">
         <v>250938</v>
       </c>
-      <c r="M49" s="38">
+      <c r="M49" s="18">
         <v>1411012</v>
       </c>
-      <c r="N49" s="38">
+      <c r="N49" s="18">
         <v>1867878</v>
       </c>
-      <c r="O49" s="38">
+      <c r="O49" s="18">
         <v>941</v>
       </c>
-      <c r="P49" s="38">
+      <c r="P49" s="18">
         <v>3102</v>
       </c>
     </row>
-    <row r="50" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A50" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="B50" s="35" t="s">
-        <v>85</v>
+    <row r="50" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A50" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>82</v>
       </c>
       <c r="C50" s="2">
         <v>57022</v>
@@ -3355,25 +3345,25 @@
         <v>71</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G50" s="2">
         <v>59</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I50" s="2">
         <v>54696</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M50" s="2">
         <v>2159</v>
@@ -3385,15 +3375,15 @@
         <v>37</v>
       </c>
       <c r="P50" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="51" spans="1:16" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A51" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="B51" s="35" t="s">
-        <v>87</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A51" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B51" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="C51" s="2">
         <v>3551423</v>
@@ -3411,7 +3401,7 @@
         <v>486</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I51" s="2">
         <v>2084793</v>
@@ -3420,10 +3410,10 @@
         <v>2992843</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M51" s="2">
         <v>1389167</v>
@@ -3438,12 +3428,12 @@
         <v>471</v>
       </c>
     </row>
-    <row r="52" spans="1:16" ht="66" x14ac:dyDescent="0.25">
-      <c r="A52" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="B52" s="35" t="s">
-        <v>89</v>
+    <row r="52" spans="1:16" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A52" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B52" s="15" t="s">
+        <v>86</v>
       </c>
       <c r="C52" s="2">
         <v>355675</v>
@@ -3488,12 +3478,12 @@
         <v>2620</v>
       </c>
     </row>
-    <row r="53" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A53" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="B53" s="35" t="s">
-        <v>91</v>
+    <row r="53" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A53" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B53" s="15" t="s">
+        <v>88</v>
       </c>
       <c r="C53" s="2">
         <v>1361</v>
@@ -3508,10 +3498,10 @@
         <v>187</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I53" s="2">
         <v>985</v>
@@ -3520,10 +3510,10 @@
         <v>599</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M53" s="2">
         <v>3</v>
@@ -3538,62 +3528,62 @@
         <v>11</v>
       </c>
     </row>
-    <row r="54" spans="1:16" s="39" customFormat="1" ht="66" x14ac:dyDescent="0.25">
-      <c r="A54" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="B54" s="40" t="s">
-        <v>92</v>
-      </c>
-      <c r="C54" s="38">
+    <row r="54" spans="1:16" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A54" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="B54" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="C54" s="18">
         <v>297296</v>
       </c>
-      <c r="D54" s="38">
+      <c r="D54" s="18">
         <v>261466</v>
       </c>
-      <c r="E54" s="38">
+      <c r="E54" s="18">
         <v>80812</v>
       </c>
-      <c r="F54" s="38">
+      <c r="F54" s="18">
         <v>141187</v>
       </c>
-      <c r="G54" s="38">
+      <c r="G54" s="18">
         <v>89</v>
       </c>
-      <c r="H54" s="38">
+      <c r="H54" s="18">
         <v>79</v>
       </c>
-      <c r="I54" s="38">
+      <c r="I54" s="18">
         <v>84345</v>
       </c>
-      <c r="J54" s="38">
+      <c r="J54" s="18">
         <v>73474</v>
       </c>
-      <c r="K54" s="38">
+      <c r="K54" s="18">
         <v>67600</v>
       </c>
-      <c r="L54" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M54" s="38">
+      <c r="L54" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="M54" s="18">
         <v>56751</v>
       </c>
-      <c r="N54" s="38">
+      <c r="N54" s="18">
         <v>14698</v>
       </c>
-      <c r="O54" s="38">
+      <c r="O54" s="18">
         <v>7699</v>
       </c>
-      <c r="P54" s="38">
+      <c r="P54" s="18">
         <v>32028</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A55" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="B55" s="35" t="s">
-        <v>94</v>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A55" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B55" s="15" t="s">
+        <v>91</v>
       </c>
       <c r="C55" s="2">
         <v>89230</v>
@@ -3602,16 +3592,16 @@
         <v>27332</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I55" s="2">
         <v>7214</v>
@@ -3623,7 +3613,7 @@
         <v>67600</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M55" s="2">
         <v>14416</v>
@@ -3632,18 +3622,18 @@
         <v>13703</v>
       </c>
       <c r="O55" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P55" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="56" spans="1:16" ht="52.8" x14ac:dyDescent="0.25">
-      <c r="A56" s="16" t="s">
-        <v>95</v>
-      </c>
-      <c r="B56" s="35" t="s">
-        <v>96</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+      <c r="A56" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B56" s="15" t="s">
+        <v>93</v>
       </c>
       <c r="C56" s="2">
         <v>6612</v>
@@ -3670,10 +3660,10 @@
         <v>15940</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M56" s="2">
         <v>352</v>
@@ -3682,18 +3672,18 @@
         <v>3</v>
       </c>
       <c r="O56" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P56" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="57" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A57" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="B57" s="35" t="s">
-        <v>98</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A57" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B57" s="15" t="s">
+        <v>95</v>
       </c>
       <c r="C57" s="2">
         <v>200601</v>
@@ -3720,10 +3710,10 @@
         <v>43456</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M57" s="2">
         <v>41527</v>
@@ -3738,12 +3728,12 @@
         <v>32028</v>
       </c>
     </row>
-    <row r="58" spans="1:16" ht="92.4" x14ac:dyDescent="0.25">
-      <c r="A58" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="B58" s="35" t="s">
-        <v>100</v>
+    <row r="58" spans="1:16" ht="89.25" x14ac:dyDescent="0.2">
+      <c r="A58" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B58" s="15" t="s">
+        <v>97</v>
       </c>
       <c r="C58" s="2">
         <v>853</v>
@@ -3758,10 +3748,10 @@
         <v>246</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I58" s="2">
         <v>151</v>
@@ -3770,10 +3760,10 @@
         <v>449</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M58" s="2">
         <v>456</v>
@@ -3782,68 +3772,68 @@
         <v>533</v>
       </c>
       <c r="O58" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P58" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="59" spans="1:16" s="39" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
-      <c r="A59" s="36" t="s">
-        <v>136</v>
-      </c>
-      <c r="B59" s="40" t="s">
-        <v>101</v>
-      </c>
-      <c r="C59" s="38">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" s="19" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A59" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="B59" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="C59" s="18">
         <v>3296</v>
       </c>
-      <c r="D59" s="38">
+      <c r="D59" s="18">
         <v>17898</v>
       </c>
-      <c r="E59" s="38">
+      <c r="E59" s="18">
         <v>2284</v>
       </c>
-      <c r="F59" s="38">
+      <c r="F59" s="18">
         <v>5072</v>
       </c>
-      <c r="G59" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="H59" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="I59" s="38">
+      <c r="G59" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="H59" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="I59" s="18">
         <v>203</v>
       </c>
-      <c r="J59" s="38">
+      <c r="J59" s="18">
         <v>578</v>
       </c>
-      <c r="K59" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="L59" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M59" s="38">
+      <c r="K59" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="L59" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="M59" s="18">
         <v>803</v>
       </c>
-      <c r="N59" s="38">
+      <c r="N59" s="18">
         <v>9036</v>
       </c>
-      <c r="O59" s="38">
+      <c r="O59" s="18">
         <v>6</v>
       </c>
-      <c r="P59" s="38">
+      <c r="P59" s="18">
         <v>3212</v>
       </c>
     </row>
-    <row r="60" spans="1:16" ht="66" x14ac:dyDescent="0.25">
-      <c r="A60" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="B60" s="35" t="s">
-        <v>103</v>
+    <row r="60" spans="1:16" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A60" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B60" s="15" t="s">
+        <v>100</v>
       </c>
       <c r="C60" s="2">
         <v>3296</v>
@@ -3858,10 +3848,10 @@
         <v>5072</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I60" s="2">
         <v>203</v>
@@ -3870,10 +3860,10 @@
         <v>578</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M60" s="2">
         <v>803</v>
@@ -3888,62 +3878,62 @@
         <v>3212</v>
       </c>
     </row>
-    <row r="61" spans="1:16" s="39" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="36" t="s">
-        <v>137</v>
-      </c>
-      <c r="B61" s="40" t="s">
-        <v>104</v>
-      </c>
-      <c r="C61" s="38">
+    <row r="61" spans="1:16" s="19" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="B61" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="C61" s="18">
         <v>929</v>
       </c>
-      <c r="D61" s="38">
+      <c r="D61" s="18">
         <v>1157</v>
       </c>
-      <c r="E61" s="38">
+      <c r="E61" s="18">
         <v>757</v>
       </c>
-      <c r="F61" s="38">
+      <c r="F61" s="18">
         <v>787</v>
       </c>
-      <c r="G61" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="H61" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="I61" s="38">
+      <c r="G61" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="H61" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="I61" s="18">
         <v>171</v>
       </c>
-      <c r="J61" s="38">
+      <c r="J61" s="18">
         <v>209</v>
       </c>
-      <c r="K61" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="L61" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M61" s="38">
+      <c r="K61" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="L61" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="M61" s="18">
         <v>1</v>
       </c>
-      <c r="N61" s="38">
+      <c r="N61" s="18">
         <v>161</v>
       </c>
-      <c r="O61" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="P61" s="38" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A62" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="B62" s="35" t="s">
-        <v>106</v>
+      <c r="O61" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="P61" s="18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A62" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="B62" s="15" t="s">
+        <v>103</v>
       </c>
       <c r="C62" s="2">
         <v>929</v>
@@ -3958,10 +3948,10 @@
         <v>787</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I62" s="2">
         <v>171</v>
@@ -3970,10 +3960,10 @@
         <v>209</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M62" s="2">
         <v>1</v>
@@ -3982,68 +3972,68 @@
         <v>161</v>
       </c>
       <c r="O62" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P62" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="63" spans="1:16" s="39" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A63" s="36" t="s">
-        <v>138</v>
-      </c>
-      <c r="B63" s="40" t="s">
-        <v>107</v>
-      </c>
-      <c r="C63" s="38">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" s="19" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A63" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="B63" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="C63" s="18">
         <v>32644</v>
       </c>
-      <c r="D63" s="38">
+      <c r="D63" s="18">
         <v>122443</v>
       </c>
-      <c r="E63" s="38">
+      <c r="E63" s="18">
         <v>1774</v>
       </c>
-      <c r="F63" s="38">
+      <c r="F63" s="18">
         <v>908</v>
       </c>
-      <c r="G63" s="38">
+      <c r="G63" s="18">
         <v>12</v>
       </c>
-      <c r="H63" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="I63" s="38">
+      <c r="H63" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="I63" s="18">
         <v>10565</v>
       </c>
-      <c r="J63" s="38">
+      <c r="J63" s="18">
         <v>90581</v>
       </c>
-      <c r="K63" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="L63" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M63" s="38">
+      <c r="K63" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="L63" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="M63" s="18">
         <v>20291</v>
       </c>
-      <c r="N63" s="38">
+      <c r="N63" s="18">
         <v>30953</v>
       </c>
-      <c r="O63" s="38">
+      <c r="O63" s="18">
         <v>2</v>
       </c>
-      <c r="P63" s="38">
+      <c r="P63" s="18">
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A64" s="16" t="s">
-        <v>108</v>
-      </c>
-      <c r="B64" s="35" t="s">
-        <v>109</v>
+    <row r="64" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A64" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B64" s="15" t="s">
+        <v>106</v>
       </c>
       <c r="C64" s="2">
         <v>31970</v>
@@ -4061,7 +4051,7 @@
         <v>12</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I64" s="2">
         <v>10414</v>
@@ -4070,10 +4060,10 @@
         <v>90430</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L64" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M64" s="2">
         <v>19780</v>
@@ -4085,15 +4075,15 @@
         <v>1</v>
       </c>
       <c r="P64" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="65" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A65" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="B65" s="35" t="s">
-        <v>111</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A65" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="B65" s="15" t="s">
+        <v>108</v>
       </c>
       <c r="C65" s="2">
         <v>674</v>
@@ -4108,10 +4098,10 @@
         <v>11</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I65" s="2">
         <v>151</v>
@@ -4120,10 +4110,10 @@
         <v>151</v>
       </c>
       <c r="K65" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L65" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M65" s="2">
         <v>511</v>
@@ -4138,62 +4128,62 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:16" s="39" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
-      <c r="A66" s="36" t="s">
-        <v>139</v>
-      </c>
-      <c r="B66" s="40" t="s">
-        <v>112</v>
-      </c>
-      <c r="C66" s="38">
+    <row r="66" spans="1:16" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A66" s="16" t="s">
+        <v>136</v>
+      </c>
+      <c r="B66" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="C66" s="18">
         <v>354</v>
       </c>
-      <c r="D66" s="38">
+      <c r="D66" s="18">
         <v>117</v>
       </c>
-      <c r="E66" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="F66" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="G66" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="H66" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="I66" s="38">
+      <c r="E66" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="F66" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="G66" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="H66" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="I66" s="18">
         <v>85</v>
       </c>
-      <c r="J66" s="38">
+      <c r="J66" s="18">
         <v>85</v>
       </c>
-      <c r="K66" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="L66" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M66" s="38">
+      <c r="K66" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="L66" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="M66" s="18">
         <v>269</v>
       </c>
-      <c r="N66" s="38">
-        <v>32</v>
-      </c>
-      <c r="O66" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="P66" s="38" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="67" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A67" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="B67" s="35" t="s">
-        <v>114</v>
+      <c r="N66" s="18">
+        <v>32</v>
+      </c>
+      <c r="O66" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="P66" s="18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A67" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B67" s="15" t="s">
+        <v>111</v>
       </c>
       <c r="C67" s="2">
         <v>354</v>
@@ -4202,16 +4192,16 @@
         <v>117</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H67" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I67" s="2">
         <v>85</v>
@@ -4220,10 +4210,10 @@
         <v>85</v>
       </c>
       <c r="K67" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L67" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M67" s="2">
         <v>269</v>
@@ -4232,68 +4222,68 @@
         <v>32</v>
       </c>
       <c r="O67" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P67" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="68" spans="1:16" s="39" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A68" s="41" t="s">
-        <v>140</v>
-      </c>
-      <c r="B68" s="42" t="s">
-        <v>115</v>
-      </c>
-      <c r="C68" s="43">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" s="19" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A68" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="B68" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C68" s="23">
         <v>500345</v>
       </c>
-      <c r="D68" s="43">
+      <c r="D68" s="23">
         <v>549868</v>
       </c>
-      <c r="E68" s="43">
+      <c r="E68" s="23">
         <v>572</v>
       </c>
-      <c r="F68" s="43">
+      <c r="F68" s="23">
         <v>280</v>
       </c>
-      <c r="G68" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="H68" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="I68" s="43">
+      <c r="G68" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="H68" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="I68" s="23">
         <v>24116</v>
       </c>
-      <c r="J68" s="43">
+      <c r="J68" s="23">
         <v>17553</v>
       </c>
-      <c r="K68" s="43">
+      <c r="K68" s="23">
         <v>32000</v>
       </c>
-      <c r="L68" s="43">
+      <c r="L68" s="23">
         <v>38800</v>
       </c>
-      <c r="M68" s="43">
+      <c r="M68" s="23">
         <v>443529</v>
       </c>
-      <c r="N68" s="43">
+      <c r="N68" s="23">
         <v>492938</v>
       </c>
-      <c r="O68" s="43">
+      <c r="O68" s="23">
         <v>128</v>
       </c>
-      <c r="P68" s="43">
+      <c r="P68" s="23">
         <v>297</v>
       </c>
     </row>
-    <row r="69" spans="1:16" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A69" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="B69" s="35" t="s">
-        <v>117</v>
+    <row r="69" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A69" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="B69" s="15" t="s">
+        <v>114</v>
       </c>
       <c r="C69" s="2">
         <v>480901</v>
@@ -4308,10 +4298,10 @@
         <v>233</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I69" s="2">
         <v>5200</v>
@@ -4338,12 +4328,12 @@
         <v>170</v>
       </c>
     </row>
-    <row r="70" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A70" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="B70" s="35" t="s">
-        <v>119</v>
+    <row r="70" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A70" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="B70" s="15" t="s">
+        <v>116</v>
       </c>
       <c r="C70" s="2">
         <v>19444</v>
@@ -4358,10 +4348,10 @@
         <v>47</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I70" s="2">
         <v>18916</v>
@@ -4370,10 +4360,10 @@
         <v>14162</v>
       </c>
       <c r="K70" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L70" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M70" s="2">
         <v>62</v>
@@ -4390,6 +4380,11 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="C2:H2"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="B5:B8"/>
+    <mergeCell ref="C5:D7"/>
     <mergeCell ref="K3:O3"/>
     <mergeCell ref="C1:H1"/>
     <mergeCell ref="E5:J5"/>
@@ -4403,11 +4398,6 @@
     <mergeCell ref="M6:N7"/>
     <mergeCell ref="O4:P4"/>
     <mergeCell ref="K5:P5"/>
-    <mergeCell ref="A5:A8"/>
-    <mergeCell ref="C2:H2"/>
-    <mergeCell ref="C3:H3"/>
-    <mergeCell ref="B5:B8"/>
-    <mergeCell ref="C5:D7"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.78740157480314965" right="0.19685039370078741" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>